<commit_message>
Fix BUG-005: alias xlsx to patched SheetJS (@e965/xlsx 0.20.3)
The npm `xlsx` package is stuck at the vulnerable 0.18.5 (prototype
pollution + ReDoS, no registry fix). Alias the dependency to the patched
SheetJS build published to npm as @e965/xlsx 0.20.3:

    "xlsx": "npm:@e965/xlsx@^0.20.3"

`import * as XLSX from 'xlsx'` is unchanged (drop-in), `npm audit` no
longer reports the xlsx advisories, 88 tests pass, and the production
build compiles. The earlier upload hardening (type/size/row caps +
try/catch) remains as defense-in-depth.

Update the QA bug report (BUG-005 -> Fixed) and change log (also records
the production RPC deploy and the real-Supabase RLS validation).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UKgs9YA8dwySKm4rWeUEMm
</commit_message>
<xml_diff>
--- a/qa-reports/04-test-cases.xlsx
+++ b/qa-reports/04-test-cases.xlsx
@@ -7,8 +7,8 @@
     <sheet name="Summary" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Test Cases'!A1:Q73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1">'Summary'!A1:B60</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Test Cases'!$A$1:$Q$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1">Summary!$A$1:$B$60</definedName>
   </definedNames>
 </workbook>
 </file>

</xml_diff>